<commit_message>
Che che che changes
</commit_message>
<xml_diff>
--- a/M400-50_data.xlsx
+++ b/M400-50_data.xlsx
@@ -53,13 +53,19 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -246,11 +252,11 @@
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="9" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -587,7 +593,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -605,7 +611,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="20.25">
       <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
@@ -623,7 +629,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="10">
         <v>0</v>
       </c>
@@ -641,7 +647,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="15">
         <v>4.673685781</v>
       </c>
@@ -659,7 +665,7 @@
         <v>0.09</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="15">
         <v>8.755577677</v>
       </c>
@@ -677,7 +683,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="15">
         <v>12.15461769</v>
       </c>
@@ -695,7 +701,7 @@
         <v>0.32</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="15">
         <v>15.07511604</v>
       </c>
@@ -713,7 +719,7 @@
         <v>0.46</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="15">
         <v>17.62449714</v>
       </c>
@@ -731,7 +737,7 @@
         <v>0.62</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="15">
         <v>19.88324558</v>
       </c>
@@ -749,7 +755,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="15">
         <v>21.90864141</v>
       </c>
@@ -767,7 +773,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="15">
         <v>23.74293655</v>
       </c>
@@ -785,7 +791,7 @@
         <v>1.22</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="15">
         <v>25.418052</v>
       </c>
@@ -803,7 +809,7 @@
         <v>1.46</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="15">
         <v>26.95865407</v>
       </c>
@@ -821,7 +827,7 @@
         <v>1.73</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="15">
         <v>28.38418164</v>
       </c>
@@ -839,7 +845,7 @@
         <v>2.04</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="15">
         <v>29.71021895</v>
       </c>
@@ -857,7 +863,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="15">
         <v>30.94944871</v>
       </c>
@@ -875,7 +881,7 @@
         <v>2.88</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
       <c r="A18" s="15">
         <v>32.11232899</v>
       </c>
@@ -893,7 +899,7 @@
         <v>3.42</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
       <c r="A19" s="15">
         <v>33.20758428</v>
       </c>
@@ -911,7 +917,7 @@
         <v>3.96</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
       <c r="A20" s="15">
         <v>34.24256843</v>
       </c>
@@ -929,7 +935,7 @@
         <v>4.38</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
       <c r="A21" s="15">
         <v>35.22353748</v>
       </c>
@@ -947,7 +953,7 @@
         <v>4.74</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
       <c r="A22" s="15">
         <v>36.15585792</v>
       </c>
@@ -959,7 +965,7 @@
       <c r="E22" s="23"/>
       <c r="F22" s="23"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
       <c r="A23" s="15">
         <v>37.04416792</v>
       </c>
@@ -971,7 +977,7 @@
       <c r="E23" s="23"/>
       <c r="F23" s="23"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5">
       <c r="A24" s="15">
         <v>37.89250362</v>
       </c>
@@ -983,7 +989,7 @@
       <c r="E24" s="23"/>
       <c r="F24" s="23"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="19.5">
       <c r="A25" s="15">
         <v>38.70439928</v>
       </c>
@@ -995,7 +1001,7 @@
       <c r="E25" s="23"/>
       <c r="F25" s="23"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="19.5">
       <c r="A26" s="15">
         <v>39.48296749</v>
       </c>

</xml_diff>